<commit_message>
Mask one internal source ID in S3 display copies with archived v1 provenance
</commit_message>
<xml_diff>
--- a/revision_artifacts/s3_paired_review50_20261019/outputs/01a13537-s3/01_仅此目录可发评审/数值候选独立评分.xlsx
+++ b/revision_artifacts/s3_paired_review50_20261019/outputs/01a13537-s3/01_仅此目录可发评审/数值候选独立评分.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="身份与说明" sheetId="1" r:id="R28376bb2af444569"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分定义" sheetId="2" r:id="R180bdcce7b394555"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分50" sheetId="3" r:id="Rd35230744f224c55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整原文" sheetId="4" r:id="R2337c9f53a4d477f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="身份与说明" sheetId="1" r:id="R73b57dade9464e5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分定义" sheetId="2" r:id="Rd7da7a9fc92d415b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分50" sheetId="3" r:id="R67b1e341a5bd4098"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整原文" sheetId="4" r:id="R7c32c082ad164f4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1689,7 +1689,7 @@
 缸套冷却出口处温度监测值在60°C至92°C范围内
 LP TC增压空气冷却器出口处温度监测标称值为90°C
 发动机进口处启动前预热温度监测值为-100°C
-温度监测参数可追溯至S30 MAN Energy Solutions 49/60 Project Guide</x:v>
+温度监测参数可追溯至 MAN Energy Solutions 49/60 Project Guide</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="16" customHeight="1">

</xml_diff>